<commit_message>
Documentation and KiCad Files changes
</commit_message>
<xml_diff>
--- a/Purchasing/BOM/BOM LIST FOC Drive Board.xlsx
+++ b/Purchasing/BOM/BOM LIST FOC Drive Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elijahrobinson/Documents/GitHub/Robot-Dog/Purchasing/BOM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FEA020D-FDEA-294E-A18C-09D5C51BA867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A5BBA3F-AF30-F847-BF8D-6077B4A7B45F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1080" yWindow="1220" windowWidth="27640" windowHeight="16620" xr2:uid="{3A4DB5C0-FC09-5F4C-A541-F46BD7668C0C}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$D$2:$D$47</definedName>
   </definedNames>
-  <calcPr calcId="191029" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -580,28 +580,22 @@
   </cellStyleXfs>
   <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -618,6 +612,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -975,1713 +975,1713 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="21" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="22" t="s">
+      <c r="C2" s="19" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="22" t="s">
+      <c r="E2" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="22" t="s">
+      <c r="F2" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="22" t="s">
+      <c r="G2" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="22" t="s">
-        <v>5</v>
-      </c>
-      <c r="I2" s="22" t="s">
+      <c r="H2" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" s="20" t="s">
         <v>118</v>
       </c>
-      <c r="J2" s="22" t="s">
+      <c r="J2" s="20" t="s">
         <v>119</v>
       </c>
-      <c r="K2" s="22" t="s">
+      <c r="K2" s="20" t="s">
         <v>116</v>
       </c>
-      <c r="L2" s="22" t="s">
+      <c r="L2" s="20" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B3" s="19">
-        <v>1</v>
-      </c>
-      <c r="C3" s="4" t="s">
+      <c r="B3" s="17">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="2">
         <v>15</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="6">
+      <c r="G3" s="4">
         <v>180</v>
       </c>
-      <c r="H3" s="6">
+      <c r="H3" s="4">
         <v>180</v>
       </c>
-      <c r="I3" s="7">
+      <c r="I3" s="5">
         <f>G3/H3</f>
         <v>1</v>
       </c>
-      <c r="J3" s="6">
+      <c r="J3" s="4">
         <f>E3*5</f>
         <v>75</v>
       </c>
-      <c r="K3" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L3" s="8" t="s">
+      <c r="K3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L3" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B4" s="19">
+      <c r="B4" s="17">
         <v>2</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" s="4">
+      <c r="D4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="2">
         <v>4</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="6">
+      <c r="G4" s="4">
         <v>48</v>
       </c>
-      <c r="H4" s="6">
+      <c r="H4" s="4">
         <v>48</v>
       </c>
-      <c r="I4" s="7">
+      <c r="I4" s="5">
         <f t="shared" ref="I4:I47" si="0">G4/H4</f>
         <v>1</v>
       </c>
-      <c r="J4" s="6">
+      <c r="J4" s="4">
         <f t="shared" ref="J4:J47" si="1">E4*5</f>
         <v>20</v>
       </c>
-      <c r="K4" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L4" s="8" t="s">
+      <c r="K4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L4" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B5" s="19">
+      <c r="B5" s="17">
         <v>3</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="2">
         <v>6</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="3">
         <v>22</v>
       </c>
-      <c r="G5" s="6">
+      <c r="G5" s="4">
         <v>72</v>
       </c>
-      <c r="H5" s="6">
+      <c r="H5" s="4">
         <v>72</v>
       </c>
-      <c r="I5" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J5" s="6">
+      <c r="I5" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J5" s="4">
         <f t="shared" si="1"/>
         <v>30</v>
       </c>
-      <c r="K5" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L5" s="8" t="s">
+      <c r="K5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L5" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="6" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B6" s="19">
+      <c r="B6" s="17">
         <v>4</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="4">
-        <v>1</v>
-      </c>
-      <c r="F6" s="5" t="s">
+      <c r="E6" s="2">
+        <v>1</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G6" s="6">
-        <v>12</v>
-      </c>
-      <c r="H6" s="6">
-        <v>12</v>
-      </c>
-      <c r="I6" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J6" s="6">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K6" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L6" s="8" t="s">
+      <c r="G6" s="4">
+        <v>12</v>
+      </c>
+      <c r="H6" s="4">
+        <v>12</v>
+      </c>
+      <c r="I6" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J6" s="4">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L6" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B7" s="19">
-        <v>5</v>
-      </c>
-      <c r="C7" s="4" t="s">
+      <c r="B7" s="17">
+        <v>5</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="4">
-        <v>1</v>
-      </c>
-      <c r="F7" s="5" t="s">
+      <c r="E7" s="2">
+        <v>1</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G7" s="6">
-        <v>12</v>
-      </c>
-      <c r="H7" s="6">
-        <v>12</v>
-      </c>
-      <c r="I7" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J7" s="6">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K7" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L7" s="8" t="s">
+      <c r="G7" s="4">
+        <v>12</v>
+      </c>
+      <c r="H7" s="4">
+        <v>12</v>
+      </c>
+      <c r="I7" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J7" s="4">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L7" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B8" s="19">
+      <c r="B8" s="17">
         <v>6</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E8" s="2">
         <v>3</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="G8" s="6">
+      <c r="G8" s="4">
         <v>36</v>
       </c>
-      <c r="H8" s="6">
+      <c r="H8" s="4">
         <v>36</v>
       </c>
-      <c r="I8" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J8" s="6">
+      <c r="I8" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J8" s="4">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="K8" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L8" s="8" t="s">
+      <c r="K8" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L8" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B9" s="19">
+      <c r="B9" s="17">
         <v>7</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E9" s="4">
-        <v>1</v>
-      </c>
-      <c r="F9" s="5" t="s">
+      <c r="E9" s="2">
+        <v>1</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="G9" s="6">
-        <v>12</v>
-      </c>
-      <c r="H9" s="6">
-        <v>12</v>
-      </c>
-      <c r="I9" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J9" s="6">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K9" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L9" s="8" t="s">
+      <c r="G9" s="4">
+        <v>12</v>
+      </c>
+      <c r="H9" s="4">
+        <v>12</v>
+      </c>
+      <c r="I9" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J9" s="4">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L9" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B10" s="19">
+      <c r="B10" s="17">
         <v>8</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="2">
         <v>3</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F10" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="G10" s="6">
+      <c r="G10" s="4">
         <v>36</v>
       </c>
-      <c r="H10" s="6">
+      <c r="H10" s="4">
         <v>36</v>
       </c>
-      <c r="I10" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J10" s="6">
+      <c r="I10" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J10" s="4">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="K10" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L10" s="8" t="s">
+      <c r="K10" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L10" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B11" s="19">
+      <c r="B11" s="17">
         <v>9</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="2">
         <v>3</v>
       </c>
-      <c r="F11" s="5" t="s">
+      <c r="F11" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="G11" s="6">
+      <c r="G11" s="4">
         <v>36</v>
       </c>
-      <c r="H11" s="6">
+      <c r="H11" s="4">
         <v>36</v>
       </c>
-      <c r="I11" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J11" s="6">
+      <c r="I11" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J11" s="4">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="K11" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L11" s="8" t="s">
+      <c r="K11" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L11" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B12" s="19">
-        <v>10</v>
-      </c>
-      <c r="C12" s="4" t="s">
+      <c r="B12" s="17">
+        <v>10</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E12" s="4">
+      <c r="E12" s="2">
         <v>2</v>
       </c>
-      <c r="F12" s="5" t="s">
+      <c r="F12" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="G12" s="6">
+      <c r="G12" s="4">
         <v>24</v>
       </c>
-      <c r="H12" s="6">
+      <c r="H12" s="4">
         <v>24</v>
       </c>
-      <c r="I12" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J12" s="6">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="K12" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L12" s="8" t="s">
+      <c r="I12" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J12" s="4">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L12" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B13" s="19">
+      <c r="B13" s="17">
         <v>11</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="E13" s="4">
-        <v>1</v>
-      </c>
-      <c r="F13" s="5" t="s">
+      <c r="E13" s="2">
+        <v>1</v>
+      </c>
+      <c r="F13" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="G13" s="6">
-        <v>12</v>
-      </c>
-      <c r="H13" s="6">
-        <v>12</v>
-      </c>
-      <c r="I13" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J13" s="6">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K13" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L13" s="8" t="s">
+      <c r="G13" s="4">
+        <v>12</v>
+      </c>
+      <c r="H13" s="4">
+        <v>12</v>
+      </c>
+      <c r="I13" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J13" s="4">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L13" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B14" s="19">
-        <v>12</v>
-      </c>
-      <c r="C14" s="9" t="s">
+      <c r="B14" s="17">
+        <v>12</v>
+      </c>
+      <c r="C14" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="D14" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="E14" s="9">
-        <v>1</v>
-      </c>
-      <c r="F14" s="10" t="s">
+      <c r="E14" s="7">
+        <v>1</v>
+      </c>
+      <c r="F14" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="G14" s="6">
-        <v>10</v>
-      </c>
-      <c r="H14" s="6">
-        <v>12</v>
-      </c>
-      <c r="I14" s="7">
+      <c r="G14" s="4">
+        <v>10</v>
+      </c>
+      <c r="H14" s="4">
+        <v>12</v>
+      </c>
+      <c r="I14" s="5">
         <f t="shared" si="0"/>
         <v>0.83333333333333337</v>
       </c>
-      <c r="J14" s="6">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K14" s="6" t="s">
+      <c r="J14" s="4">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K14" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="L14" s="8" t="s">
+      <c r="L14" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B15" s="19">
+      <c r="B15" s="17">
         <v>13</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="D15" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="E15" s="9">
-        <v>1</v>
-      </c>
-      <c r="F15" s="10" t="s">
+      <c r="E15" s="7">
+        <v>1</v>
+      </c>
+      <c r="F15" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="G15" s="6">
-        <v>10</v>
-      </c>
-      <c r="H15" s="6">
-        <v>12</v>
-      </c>
-      <c r="I15" s="7">
+      <c r="G15" s="4">
+        <v>10</v>
+      </c>
+      <c r="H15" s="4">
+        <v>12</v>
+      </c>
+      <c r="I15" s="5">
         <f t="shared" si="0"/>
         <v>0.83333333333333337</v>
       </c>
-      <c r="J15" s="6">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K15" s="6" t="s">
+      <c r="J15" s="4">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K15" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="L15" s="8" t="s">
+      <c r="L15" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B16" s="19">
+      <c r="B16" s="17">
         <v>14</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="E16" s="4">
+      <c r="E16" s="2">
         <v>2</v>
       </c>
-      <c r="F16" s="5" t="s">
+      <c r="F16" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="G16" s="6">
+      <c r="G16" s="4">
         <v>24</v>
       </c>
-      <c r="H16" s="6">
+      <c r="H16" s="4">
         <v>24</v>
       </c>
-      <c r="I16" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J16" s="6">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="K16" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L16" s="8" t="s">
+      <c r="I16" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J16" s="4">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="K16" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L16" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="17" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B17" s="19">
+      <c r="B17" s="17">
         <v>15</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E17" s="4">
+      <c r="E17" s="2">
         <v>2</v>
       </c>
-      <c r="F17" s="5">
+      <c r="F17" s="3">
         <v>0</v>
       </c>
-      <c r="G17" s="6">
+      <c r="G17" s="4">
         <v>24</v>
       </c>
-      <c r="H17" s="6">
+      <c r="H17" s="4">
         <v>24</v>
       </c>
-      <c r="I17" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J17" s="6">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="K17" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L17" s="8" t="s">
+      <c r="I17" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J17" s="4">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="K17" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L17" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B18" s="19">
+      <c r="B18" s="17">
         <v>16</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C18" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="D18" s="9" t="s">
+      <c r="D18" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="E18" s="9">
+      <c r="E18" s="7">
         <v>6</v>
       </c>
-      <c r="F18" s="10" t="s">
+      <c r="F18" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="G18" s="6">
+      <c r="G18" s="4">
         <v>30</v>
       </c>
-      <c r="H18" s="6">
+      <c r="H18" s="4">
         <v>72</v>
       </c>
-      <c r="I18" s="7">
+      <c r="I18" s="5">
         <f t="shared" si="0"/>
         <v>0.41666666666666669</v>
       </c>
-      <c r="J18" s="6">
+      <c r="J18" s="4">
         <f t="shared" si="1"/>
         <v>30</v>
       </c>
-      <c r="K18" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L18" s="8" t="s">
+      <c r="K18" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L18" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B19" s="19">
+      <c r="B19" s="17">
         <v>17</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E19" s="4">
-        <v>1</v>
-      </c>
-      <c r="F19" s="5">
+      <c r="E19" s="2">
+        <v>1</v>
+      </c>
+      <c r="F19" s="3">
         <v>0</v>
       </c>
-      <c r="G19" s="6">
-        <v>12</v>
-      </c>
-      <c r="H19" s="6">
-        <v>12</v>
-      </c>
-      <c r="I19" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J19" s="6">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K19" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L19" s="8" t="s">
+      <c r="G19" s="4">
+        <v>12</v>
+      </c>
+      <c r="H19" s="4">
+        <v>12</v>
+      </c>
+      <c r="I19" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J19" s="4">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K19" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L19" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B20" s="19">
+      <c r="B20" s="17">
         <v>18</v>
       </c>
-      <c r="C20" s="11" t="s">
+      <c r="C20" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="D20" s="11" t="s">
+      <c r="D20" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="E20" s="11">
-        <v>1</v>
-      </c>
-      <c r="F20" s="12" t="s">
+      <c r="E20" s="9">
+        <v>1</v>
+      </c>
+      <c r="F20" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="G20" s="6">
-        <v>12</v>
-      </c>
-      <c r="H20" s="6">
-        <v>12</v>
-      </c>
-      <c r="I20" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J20" s="6">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K20" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L20" s="8" t="s">
+      <c r="G20" s="4">
+        <v>12</v>
+      </c>
+      <c r="H20" s="4">
+        <v>12</v>
+      </c>
+      <c r="I20" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J20" s="4">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K20" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L20" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B21" s="19">
+      <c r="B21" s="17">
         <v>19</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="E21" s="4">
-        <v>1</v>
-      </c>
-      <c r="F21" s="5" t="s">
+      <c r="E21" s="7">
+        <v>1</v>
+      </c>
+      <c r="F21" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="G21" s="6">
-        <v>12</v>
-      </c>
-      <c r="H21" s="6">
-        <v>12</v>
-      </c>
-      <c r="I21" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J21" s="6">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K21" s="6" t="s">
+      <c r="G21" s="4">
+        <v>10</v>
+      </c>
+      <c r="H21" s="4">
+        <v>12</v>
+      </c>
+      <c r="I21" s="5">
+        <f t="shared" si="0"/>
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="J21" s="4">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K21" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="L21" s="8" t="s">
+      <c r="L21" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B22" s="19">
+      <c r="B22" s="17">
         <v>20</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E22" s="4">
+      <c r="E22" s="2">
         <v>3</v>
       </c>
-      <c r="F22" s="5" t="s">
+      <c r="F22" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="G22" s="6">
+      <c r="G22" s="4">
         <v>36</v>
       </c>
-      <c r="H22" s="6">
+      <c r="H22" s="4">
         <v>36</v>
       </c>
-      <c r="I22" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J22" s="6">
+      <c r="I22" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J22" s="4">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="K22" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L22" s="8" t="s">
+      <c r="K22" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L22" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="23" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B23" s="19">
+      <c r="B23" s="17">
         <v>21</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D23" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E23" s="4">
-        <v>1</v>
-      </c>
-      <c r="F23" s="5" t="s">
+      <c r="E23" s="2">
+        <v>1</v>
+      </c>
+      <c r="F23" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="G23" s="6">
-        <v>12</v>
-      </c>
-      <c r="H23" s="6">
-        <v>12</v>
-      </c>
-      <c r="I23" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J23" s="6">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K23" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L23" s="8" t="s">
+      <c r="G23" s="4">
+        <v>12</v>
+      </c>
+      <c r="H23" s="4">
+        <v>12</v>
+      </c>
+      <c r="I23" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J23" s="4">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K23" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L23" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B24" s="19">
+      <c r="B24" s="17">
         <v>22</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D24" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="E24" s="4">
+      <c r="E24" s="2">
         <v>2</v>
       </c>
-      <c r="F24" s="5" t="s">
+      <c r="F24" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="G24" s="6">
+      <c r="G24" s="4">
         <v>24</v>
       </c>
-      <c r="H24" s="6">
+      <c r="H24" s="4">
         <v>24</v>
       </c>
-      <c r="I24" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J24" s="6">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="K24" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L24" s="8" t="s">
+      <c r="I24" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J24" s="4">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="K24" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L24" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B25" s="19">
+      <c r="B25" s="17">
         <v>23</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="D25" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E25" s="4">
-        <v>1</v>
-      </c>
-      <c r="F25" s="5" t="s">
+      <c r="E25" s="2">
+        <v>1</v>
+      </c>
+      <c r="F25" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="G25" s="6">
-        <v>12</v>
-      </c>
-      <c r="H25" s="6">
-        <v>12</v>
-      </c>
-      <c r="I25" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J25" s="6">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K25" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L25" s="8" t="s">
+      <c r="G25" s="4">
+        <v>12</v>
+      </c>
+      <c r="H25" s="4">
+        <v>12</v>
+      </c>
+      <c r="I25" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J25" s="4">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K25" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L25" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B26" s="19">
+      <c r="B26" s="17">
         <v>24</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="C26" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="D26" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E26" s="4">
+      <c r="E26" s="2">
         <v>2</v>
       </c>
-      <c r="F26" s="5" t="s">
+      <c r="F26" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="G26" s="6">
+      <c r="G26" s="4">
         <v>24</v>
       </c>
-      <c r="H26" s="6">
+      <c r="H26" s="4">
         <v>24</v>
       </c>
-      <c r="I26" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J26" s="6">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="K26" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L26" s="8" t="s">
+      <c r="I26" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J26" s="4">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="K26" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L26" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="27" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B27" s="19">
+      <c r="B27" s="17">
         <v>25</v>
       </c>
-      <c r="C27" s="9" t="s">
+      <c r="C27" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="D27" s="9" t="s">
+      <c r="D27" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="E27" s="9">
+      <c r="E27" s="7">
         <v>2</v>
       </c>
-      <c r="F27" s="10" t="s">
+      <c r="F27" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="G27" s="6">
-        <v>5</v>
-      </c>
-      <c r="H27" s="6">
+      <c r="G27" s="4">
+        <v>5</v>
+      </c>
+      <c r="H27" s="4">
         <v>24</v>
       </c>
-      <c r="I27" s="7">
+      <c r="I27" s="5">
         <f t="shared" si="0"/>
         <v>0.20833333333333334</v>
       </c>
-      <c r="J27" s="6">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="K27" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L27" s="8" t="s">
+      <c r="J27" s="4">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="K27" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L27" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="28" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B28" s="19">
+      <c r="B28" s="17">
         <v>26</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="C28" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="D28" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E28" s="4">
+      <c r="E28" s="2">
         <v>3</v>
       </c>
-      <c r="F28" s="5" t="s">
+      <c r="F28" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="G28" s="6">
+      <c r="G28" s="4">
         <v>36</v>
       </c>
-      <c r="H28" s="6">
+      <c r="H28" s="4">
         <v>36</v>
       </c>
-      <c r="I28" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J28" s="6">
+      <c r="I28" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J28" s="4">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="K28" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L28" s="8" t="s">
+      <c r="K28" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L28" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="29" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B29" s="19">
+      <c r="B29" s="17">
         <v>27</v>
       </c>
-      <c r="C29" s="4" t="s">
+      <c r="C29" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D29" s="4" t="s">
+      <c r="D29" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E29" s="4">
+      <c r="E29" s="2">
         <v>3</v>
       </c>
-      <c r="F29" s="5" t="s">
+      <c r="F29" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="G29" s="6">
+      <c r="G29" s="4">
         <v>36</v>
       </c>
-      <c r="H29" s="6">
+      <c r="H29" s="4">
         <v>36</v>
       </c>
-      <c r="I29" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J29" s="6">
+      <c r="I29" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J29" s="4">
         <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="K29" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L29" s="8" t="s">
+      <c r="K29" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L29" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="30" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B30" s="19">
+      <c r="B30" s="17">
         <v>28</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="C30" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="D30" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E30" s="4">
+      <c r="D30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E30" s="2">
         <v>2</v>
       </c>
-      <c r="F30" s="5" t="s">
+      <c r="F30" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="G30" s="6">
+      <c r="G30" s="4">
         <v>24</v>
       </c>
-      <c r="H30" s="6">
+      <c r="H30" s="4">
         <v>24</v>
       </c>
-      <c r="I30" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J30" s="6">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="K30" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L30" s="8" t="s">
+      <c r="I30" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J30" s="4">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="K30" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L30" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B31" s="19">
+      <c r="B31" s="17">
         <v>29</v>
       </c>
-      <c r="C31" s="9" t="s">
+      <c r="C31" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="D31" s="9" t="s">
+      <c r="D31" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="E31" s="9">
-        <v>1</v>
-      </c>
-      <c r="F31" s="10" t="s">
+      <c r="E31" s="7">
+        <v>1</v>
+      </c>
+      <c r="F31" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="G31" s="6">
-        <v>10</v>
-      </c>
-      <c r="H31" s="6">
-        <v>12</v>
-      </c>
-      <c r="I31" s="7">
+      <c r="G31" s="4">
+        <v>10</v>
+      </c>
+      <c r="H31" s="4">
+        <v>12</v>
+      </c>
+      <c r="I31" s="5">
         <f t="shared" si="0"/>
         <v>0.83333333333333337</v>
       </c>
-      <c r="J31" s="6">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K31" s="6" t="s">
+      <c r="J31" s="4">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K31" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="L31" s="8" t="s">
+      <c r="L31" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="32" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B32" s="19">
+      <c r="B32" s="17">
         <v>30</v>
       </c>
-      <c r="C32" s="4" t="s">
+      <c r="C32" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="D32" s="4" t="s">
+      <c r="D32" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E32" s="4">
-        <v>1</v>
-      </c>
-      <c r="F32" s="5" t="s">
+      <c r="E32" s="2">
+        <v>1</v>
+      </c>
+      <c r="F32" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="G32" s="6">
-        <v>12</v>
-      </c>
-      <c r="H32" s="6">
-        <v>12</v>
-      </c>
-      <c r="I32" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J32" s="6">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K32" s="6" t="s">
+      <c r="G32" s="4">
+        <v>12</v>
+      </c>
+      <c r="H32" s="4">
+        <v>12</v>
+      </c>
+      <c r="I32" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J32" s="4">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K32" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="L32" s="8" t="s">
+      <c r="L32" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="33" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B33" s="19">
+      <c r="B33" s="17">
         <v>31</v>
       </c>
-      <c r="C33" s="4" t="s">
+      <c r="C33" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="D33" s="4" t="s">
+      <c r="D33" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E33" s="4">
+      <c r="E33" s="2">
         <v>2</v>
       </c>
-      <c r="F33" s="5" t="s">
+      <c r="F33" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="G33" s="6">
+      <c r="G33" s="4">
         <v>24</v>
       </c>
-      <c r="H33" s="6">
+      <c r="H33" s="4">
         <v>24</v>
       </c>
-      <c r="I33" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J33" s="6">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="K33" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L33" s="8" t="s">
+      <c r="I33" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J33" s="4">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="K33" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L33" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="34" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B34" s="19">
+      <c r="B34" s="17">
         <v>32</v>
       </c>
-      <c r="C34" s="4" t="s">
+      <c r="C34" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="D34" s="4" t="s">
+      <c r="D34" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="E34" s="4">
-        <v>1</v>
-      </c>
-      <c r="F34" s="5" t="s">
+      <c r="E34" s="2">
+        <v>1</v>
+      </c>
+      <c r="F34" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="G34" s="6">
-        <v>12</v>
-      </c>
-      <c r="H34" s="6">
-        <v>12</v>
-      </c>
-      <c r="I34" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J34" s="6">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K34" s="6" t="s">
+      <c r="G34" s="4">
+        <v>12</v>
+      </c>
+      <c r="H34" s="4">
+        <v>12</v>
+      </c>
+      <c r="I34" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J34" s="4">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K34" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="L34" s="8" t="s">
+      <c r="L34" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="35" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B35" s="19">
+      <c r="B35" s="17">
         <v>33</v>
       </c>
-      <c r="C35" s="4" t="s">
+      <c r="C35" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="D35" s="4" t="s">
+      <c r="D35" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="E35" s="4">
-        <v>1</v>
-      </c>
-      <c r="F35" s="5" t="s">
+      <c r="E35" s="2">
+        <v>1</v>
+      </c>
+      <c r="F35" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="G35" s="6">
+      <c r="G35" s="4">
         <v>6</v>
       </c>
-      <c r="H35" s="6">
-        <v>12</v>
-      </c>
-      <c r="I35" s="7">
+      <c r="H35" s="4">
+        <v>12</v>
+      </c>
+      <c r="I35" s="5">
         <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
-      <c r="J35" s="6">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K35" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L35" s="8" t="s">
+      <c r="J35" s="4">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K35" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L35" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="36" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B36" s="19">
+      <c r="B36" s="17">
         <v>34</v>
       </c>
-      <c r="C36" s="4" t="s">
+      <c r="C36" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="D36" s="4" t="s">
+      <c r="D36" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E36" s="4">
-        <v>1</v>
-      </c>
-      <c r="F36" s="5" t="s">
+      <c r="E36" s="2">
+        <v>1</v>
+      </c>
+      <c r="F36" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="G36" s="6">
-        <v>12</v>
-      </c>
-      <c r="H36" s="6">
-        <v>12</v>
-      </c>
-      <c r="I36" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J36" s="6">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K36" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L36" s="8" t="s">
+      <c r="G36" s="4">
+        <v>12</v>
+      </c>
+      <c r="H36" s="4">
+        <v>12</v>
+      </c>
+      <c r="I36" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J36" s="4">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K36" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L36" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="37" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B37" s="19">
+      <c r="B37" s="17">
         <v>35</v>
       </c>
-      <c r="C37" s="9" t="s">
+      <c r="C37" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="D37" s="9" t="s">
+      <c r="D37" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="E37" s="9">
-        <v>1</v>
-      </c>
-      <c r="F37" s="10" t="s">
+      <c r="E37" s="7">
+        <v>1</v>
+      </c>
+      <c r="F37" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="G37" s="6">
-        <v>10</v>
-      </c>
-      <c r="H37" s="6">
-        <v>12</v>
-      </c>
-      <c r="I37" s="7">
+      <c r="G37" s="4">
+        <v>10</v>
+      </c>
+      <c r="H37" s="4">
+        <v>12</v>
+      </c>
+      <c r="I37" s="5">
         <f t="shared" si="0"/>
         <v>0.83333333333333337</v>
       </c>
-      <c r="J37" s="6">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K37" s="6" t="s">
+      <c r="J37" s="4">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K37" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="L37" s="8" t="s">
+      <c r="L37" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="38" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B38" s="19">
+      <c r="B38" s="17">
         <v>36</v>
       </c>
-      <c r="C38" s="9" t="s">
+      <c r="C38" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="D38" s="9" t="s">
+      <c r="D38" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="E38" s="9">
-        <v>1</v>
-      </c>
-      <c r="F38" s="10" t="s">
+      <c r="E38" s="7">
+        <v>1</v>
+      </c>
+      <c r="F38" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="G38" s="6">
-        <v>10</v>
-      </c>
-      <c r="H38" s="6">
-        <v>12</v>
-      </c>
-      <c r="I38" s="7">
+      <c r="G38" s="4">
+        <v>10</v>
+      </c>
+      <c r="H38" s="4">
+        <v>12</v>
+      </c>
+      <c r="I38" s="5">
         <f t="shared" si="0"/>
         <v>0.83333333333333337</v>
       </c>
-      <c r="J38" s="6">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K38" s="6" t="s">
+      <c r="J38" s="4">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K38" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="L38" s="8" t="s">
+      <c r="L38" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="39" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B39" s="19">
+      <c r="B39" s="17">
         <v>37</v>
       </c>
-      <c r="C39" s="4" t="s">
+      <c r="C39" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="D39" s="4" t="s">
+      <c r="D39" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="E39" s="4">
-        <v>1</v>
-      </c>
-      <c r="F39" s="5" t="s">
+      <c r="E39" s="2">
+        <v>1</v>
+      </c>
+      <c r="F39" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G39" s="6">
-        <v>12</v>
-      </c>
-      <c r="H39" s="6">
-        <v>12</v>
-      </c>
-      <c r="I39" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J39" s="6">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K39" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L39" s="8" t="s">
+      <c r="G39" s="4">
+        <v>12</v>
+      </c>
+      <c r="H39" s="4">
+        <v>12</v>
+      </c>
+      <c r="I39" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J39" s="4">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K39" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L39" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="40" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B40" s="19">
+      <c r="B40" s="17">
         <v>38</v>
       </c>
-      <c r="C40" s="4" t="s">
+      <c r="C40" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="D40" s="4" t="s">
+      <c r="D40" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E40" s="4">
+      <c r="E40" s="2">
         <v>2</v>
       </c>
-      <c r="F40" s="5" t="s">
+      <c r="F40" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="G40" s="6">
+      <c r="G40" s="4">
         <v>24</v>
       </c>
-      <c r="H40" s="6">
+      <c r="H40" s="4">
         <v>24</v>
       </c>
-      <c r="I40" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J40" s="6">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="K40" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L40" s="8" t="s">
+      <c r="I40" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J40" s="4">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="K40" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L40" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="41" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B41" s="19">
+      <c r="B41" s="17">
         <v>39</v>
       </c>
-      <c r="C41" s="4" t="s">
+      <c r="C41" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="D41" s="4" t="s">
+      <c r="D41" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E41" s="4">
-        <v>1</v>
-      </c>
-      <c r="F41" s="5" t="s">
+      <c r="E41" s="2">
+        <v>1</v>
+      </c>
+      <c r="F41" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="G41" s="6">
-        <v>12</v>
-      </c>
-      <c r="H41" s="6">
-        <v>12</v>
-      </c>
-      <c r="I41" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J41" s="6">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K41" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L41" s="8" t="s">
+      <c r="G41" s="4">
+        <v>12</v>
+      </c>
+      <c r="H41" s="4">
+        <v>12</v>
+      </c>
+      <c r="I41" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J41" s="4">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K41" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L41" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="42" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B42" s="19">
+      <c r="B42" s="17">
         <v>40</v>
       </c>
-      <c r="C42" s="4" t="s">
+      <c r="C42" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="D42" s="4" t="s">
+      <c r="D42" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="E42" s="4">
-        <v>1</v>
-      </c>
-      <c r="F42" s="5" t="s">
+      <c r="E42" s="2">
+        <v>1</v>
+      </c>
+      <c r="F42" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="G42" s="6">
-        <v>12</v>
-      </c>
-      <c r="H42" s="6">
-        <v>12</v>
-      </c>
-      <c r="I42" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J42" s="6">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K42" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L42" s="8" t="s">
+      <c r="G42" s="4">
+        <v>12</v>
+      </c>
+      <c r="H42" s="4">
+        <v>12</v>
+      </c>
+      <c r="I42" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J42" s="4">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K42" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L42" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="43" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B43" s="19">
-        <v>41</v>
-      </c>
-      <c r="C43" s="4" t="s">
+      <c r="B43" s="17">
+        <v>41</v>
+      </c>
+      <c r="C43" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="D43" s="4" t="s">
+      <c r="D43" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="E43" s="4">
-        <v>1</v>
-      </c>
-      <c r="F43" s="5" t="s">
+      <c r="E43" s="2">
+        <v>1</v>
+      </c>
+      <c r="F43" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="G43" s="6">
-        <v>12</v>
-      </c>
-      <c r="H43" s="6">
-        <v>12</v>
-      </c>
-      <c r="I43" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J43" s="6">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K43" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L43" s="8" t="s">
+      <c r="G43" s="4">
+        <v>12</v>
+      </c>
+      <c r="H43" s="4">
+        <v>12</v>
+      </c>
+      <c r="I43" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J43" s="4">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K43" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L43" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="44" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B44" s="19">
+      <c r="B44" s="17">
         <v>42</v>
       </c>
-      <c r="C44" s="4" t="s">
+      <c r="C44" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="D44" s="4" t="s">
+      <c r="D44" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="E44" s="4">
-        <v>1</v>
-      </c>
-      <c r="F44" s="5" t="s">
+      <c r="E44" s="2">
+        <v>1</v>
+      </c>
+      <c r="F44" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="G44" s="6">
-        <v>12</v>
-      </c>
-      <c r="H44" s="6">
-        <v>12</v>
-      </c>
-      <c r="I44" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J44" s="6">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K44" s="6" t="s">
+      <c r="G44" s="4">
+        <v>12</v>
+      </c>
+      <c r="H44" s="4">
+        <v>12</v>
+      </c>
+      <c r="I44" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J44" s="4">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K44" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="L44" s="8" t="s">
+      <c r="L44" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="45" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B45" s="19">
+      <c r="B45" s="17">
         <v>43</v>
       </c>
-      <c r="C45" s="4" t="s">
+      <c r="C45" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D45" s="4" t="s">
+      <c r="D45" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="E45" s="4">
-        <v>1</v>
-      </c>
-      <c r="F45" s="5" t="s">
+      <c r="E45" s="2">
+        <v>1</v>
+      </c>
+      <c r="F45" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G45" s="6">
-        <v>12</v>
-      </c>
-      <c r="H45" s="6">
-        <v>12</v>
-      </c>
-      <c r="I45" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J45" s="6">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K45" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L45" s="8" t="s">
+      <c r="G45" s="4">
+        <v>12</v>
+      </c>
+      <c r="H45" s="4">
+        <v>12</v>
+      </c>
+      <c r="I45" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J45" s="4">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K45" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L45" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="46" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B46" s="19">
+      <c r="B46" s="17">
         <v>44</v>
       </c>
-      <c r="C46" s="4" t="s">
+      <c r="C46" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D46" s="4" t="s">
+      <c r="D46" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E46" s="4">
-        <v>1</v>
-      </c>
-      <c r="F46" s="5" t="s">
+      <c r="E46" s="2">
+        <v>1</v>
+      </c>
+      <c r="F46" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="G46" s="6">
-        <v>12</v>
-      </c>
-      <c r="H46" s="6">
-        <v>12</v>
-      </c>
-      <c r="I46" s="7">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="J46" s="6">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K46" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="L46" s="8" t="s">
+      <c r="G46" s="4">
+        <v>12</v>
+      </c>
+      <c r="H46" s="4">
+        <v>12</v>
+      </c>
+      <c r="I46" s="5">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J46" s="4">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K46" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L46" s="6" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="47" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B47" s="20">
+      <c r="B47" s="18">
         <v>45</v>
       </c>
-      <c r="C47" s="13" t="s">
+      <c r="C47" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="D47" s="13" t="s">
+      <c r="D47" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="E47" s="13">
-        <v>1</v>
-      </c>
-      <c r="F47" s="14" t="s">
+      <c r="E47" s="11">
+        <v>1</v>
+      </c>
+      <c r="F47" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="G47" s="15">
-        <v>10</v>
-      </c>
-      <c r="H47" s="15">
-        <v>12</v>
-      </c>
-      <c r="I47" s="16">
+      <c r="G47" s="13">
+        <v>10</v>
+      </c>
+      <c r="H47" s="13">
+        <v>12</v>
+      </c>
+      <c r="I47" s="14">
         <f t="shared" si="0"/>
         <v>0.83333333333333337</v>
       </c>
-      <c r="J47" s="15">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="K47" s="15" t="s">
+      <c r="J47" s="13">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K47" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="L47" s="17" t="s">
+      <c r="L47" s="15" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="50" spans="7:9" x14ac:dyDescent="0.2">
-      <c r="G50" s="1" t="s">
+      <c r="G50" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="H50" s="2"/>
-      <c r="I50" s="3">
+      <c r="H50" s="22"/>
+      <c r="I50" s="1">
         <f>SUM(I3:I47)/COUNT(I3:I47)</f>
-        <v>0.93611111111111123</v>
+        <v>0.93240740740740746</v>
       </c>
     </row>
   </sheetData>

</xml_diff>